<commit_message>
Soumission #158 : Maltese Technologies [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$286</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$286</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$287</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$287</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M286"/>
+  <dimension ref="A1:M287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4517,7 +4517,7 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>https://www.cyberium.io/</t>
+          <t>https://cyberium.io/contact/</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -19742,8 +19742,79 @@
         </is>
       </c>
     </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>Maltese Technologies</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>Préparez, gérez et anticipez vos crises en toute simplicité grâce à notre plateforme tout-en-un, optimisée pour la coordination, le suivi et les RetEx. Maltese Technologies développe des logiciels intuitifs pour aider les organisations à gérer les crises et garantir la continuité des activités. Membre d'Hexatrust, Maltese Technologies est certifié ISO27001 et propose un hébergement qualifié SecNumCloud.</t>
+        </is>
+      </c>
+      <c r="D287" s="3" t="inlineStr">
+        <is>
+          <t>Maltese Technologies développe des logiciels intuitifs pour aider les organisations à gérer les crises et garantir la continuité des activités. Nous avons créé une solution tout-en-un et collaborative qui vous permet de gagner du temps, de collaborer efficacement même sous pression, et de garder le contrôle en toutes circonstances. Membre d'Hexatrust, Maltese Technologies est certifié ISO27001 et propose un hébergement qualifié SecNumCloud. Les autres acteurs du secteur sont easylience, F24, cristotech, chapsvision, crisebox, panicsafe, iremos.
+Notre solution permet de : Gagnez du temps sur vos rapports au décideur. Rédigez et envoyez facilement vos points de situation. Publiez les mises à jour au fil de vos événements. Conservez un journal de bord. Suivez facilement les actions critiques. Gérez efficacement le temps grâce à une vue complète. Facilitez les passations d’équipes. Visualisez l’impact d’une perte critique sur vos activités. Anticipez les missions prioritaires à relancer. Orchestrez le redémarrage en identifiant les ressources clés. Pour votre main courante, vos plans de continuité, vos bilans d’analyse d’impacts… un mur de données paramétrable pour refléter votre méthodologie de résilience. Editable en équipe et en temps réel pour que vous puissiez distribuer plusieurs rôles de secrétaire et ne plus perdre d’informations.
+Nos clients: OIV administration, service public, sécurité intérieure, acteurs de l'événementiel.</t>
+        </is>
+      </c>
+      <c r="E287" s="3" t="inlineStr"/>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>RS : Répondre</t>
+        </is>
+      </c>
+      <c r="G287" s="3" t="inlineStr">
+        <is>
+          <t>RS.MA : Gestion des incidents
+PR.AT : Sensibilisation et formation
+RC.RP : Exécution du plan de reprise</t>
+        </is>
+      </c>
+      <c r="H287" s="3" t="inlineStr">
+        <is>
+          <t>RC.RP-06 : La fin de la reprise d'incident est déclarée selon des critères, avec documentation complétée
+RC.RP-02 : Les actions de reprise sont sélectionnées, cadrées, priorisées et exécutées
+RS.MA-05 : Les critères de déclenchement de la reprise d'incident sont appliqués
+RC.RP-01 : La partie reprise du plan de réponse aux incidents est exécutée une fois déclenchée
+RS.MA-03 : Les incidents sont catégorisés et priorisés</t>
+        </is>
+      </c>
+      <c r="I287" s="3" t="inlineStr">
+        <is>
+          <t>Continuité et reprise d'activité</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>https://www.maltese.tech</t>
+        </is>
+      </c>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>contact@maltese.tech</t>
+        </is>
+      </c>
+      <c r="L287" s="2" t="inlineStr">
+        <is>
+          <t>maltese-technologies.svg</t>
+        </is>
+      </c>
+      <c r="M287" s="2" t="inlineStr">
+        <is>
+          <t>maltese-technologies</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M286"/>
+  <autoFilter ref="A1:M287"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25000,7 +25071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J286"/>
+  <dimension ref="A1:J287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -39063,8 +39134,46 @@
       <c r="I286" s="3" t="inlineStr"/>
       <c r="J286" s="3" t="inlineStr"/>
     </row>
+    <row r="287">
+      <c r="A287" s="3" t="inlineStr">
+        <is>
+          <t>Maltese Technologies</t>
+        </is>
+      </c>
+      <c r="B287" s="3" t="inlineStr">
+        <is>
+          <t>RS : Répondre</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>RS.MA : Gestion des incidents
+PR.AT : Sensibilisation et formation
+RC.RP : Exécution du plan de reprise</t>
+        </is>
+      </c>
+      <c r="D287" s="3" t="inlineStr">
+        <is>
+          <t>RC.RP-06 : La fin de la reprise d'incident est déclarée selon des critères, avec documentation complétée
+RC.RP-02 : Les actions de reprise sont sélectionnées, cadrées, priorisées et exécutées
+RS.MA-05 : Les critères de déclenchement de la reprise d'incident sont appliqués
+RC.RP-01 : La partie reprise du plan de réponse aux incidents est exécutée une fois déclenchée
+RS.MA-03 : Les incidents sont catégorisés et priorisés</t>
+        </is>
+      </c>
+      <c r="E287" s="3" t="inlineStr"/>
+      <c r="F287" s="3" t="inlineStr"/>
+      <c r="G287" s="3" t="inlineStr"/>
+      <c r="H287" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I287" s="3" t="inlineStr"/>
+      <c r="J287" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J286"/>
+  <autoFilter ref="A1:J287"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #159 : NetExplorer (NetExplorer Share) [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -10115,7 +10115,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>NetExplorer (NetExplorer Share)</t>
+          <t>Voltn</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -10125,7 +10125,9 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>NetExplorer, éditeur basé à Toulouse, propose une plateforme de stockage et de partage de fichiers hébergée en France. L'offre réunit NetExplorer Share pour l'envoi sécurisé de documents, NetExplorer Workspace pour la coédition collaborative, la DataRoom pour les documents confidentiels, ainsi que les options Sign, Private Cloud, Vault sur bande LTO et hébergement HDS. La société annonce plus de 1 800 clients dans la santé, le juridique, l'immobilier, la banque et le secteur public.</t>
+          <t>Voltn (anciennement NetExplorer) est l'expert du fichier en entreprise. Stocker, partager, coéditer, signer, valider, tracer, retrouver : Voltn couvre le cycle de vie complet du fichier sans rien imposer.
+Depuis plus de quinze ans, il répond à ce besoin avec deux produits : Voltn Share pour partager avec l'extérieur, Voltn Workspace pour réunir et maîtriser les fichiers de l'entreprise.
+2 000 organisations et 300 000 utilisateurs quotidiens lui confient leurs fichiers, soit plus de 500 millions de fichiers à ce jour. L'entreprise, basée à Toulouse, héberge ces fichiers en France ou au Luxembourg. Elle est certifiée ISO 9001, ISO 27001, Hébergeur de Données de Santé (HDS) et labellisée Numérique Responsable (NR).</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
@@ -10163,17 +10165,17 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>https://www.netexplorer.fr</t>
+          <t>https://www.voltn.eu</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
         <is>
-          <t>contact@netexplorer.fr</t>
+          <t>contact@voltn.eu</t>
         </is>
       </c>
       <c r="L145" s="2" t="inlineStr">
         <is>
-          <t>NetExplorer_01.png</t>
+          <t>netexplorer-netexplorer-share.png</t>
         </is>
       </c>
       <c r="M145" s="2" t="inlineStr">
@@ -32207,7 +32209,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>NetExplorer (NetExplorer Share)</t>
+          <t>Voltn</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">

</xml_diff>